<commit_message>
update tool to use updated metadata when calculating metrics, run the tool
</commit_message>
<xml_diff>
--- a/2_calculated_metrics/gbls_corpus_metrics/gbls_feature_overview.xlsx
+++ b/2_calculated_metrics/gbls_corpus_metrics/gbls_feature_overview.xlsx
@@ -20,22 +20,28 @@
     <sheet name="Service_Area" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Audience" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Intended_Outcome" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Coding_Confidence" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Evidence_Confidence" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Service_Conditions_Addressed" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Conceptual_Theme" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Coding_Confidence" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Year Counts'!$A$1:$C$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Feature Counts'!$A$1:$F$88</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Data Dictionary'!$A$1:$C$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Source_Type'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Feature Counts'!$A$1:$F$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Data Dictionary'!$A$1:$C$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Source_Type'!$A$1:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Peer_Review'!$A$1:$E$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Evidence_Type'!$A$1:$E$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Primary_Methodology'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Evidence_Type'!$A$1:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Primary_Methodology'!$A$1:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Library_Context'!$A$1:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Game_Format'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Service_Area'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Audience'!$A$1:$E$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Intended_Outcome'!$A$1:$E$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Coding_Confidence'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Game_Format'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Service_Area'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Audience'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Intended_Outcome'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Evidence_Confidence'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Service_Conditions_Addressed'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Conceptual_Theme'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Coding_Confidence'!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -491,7 +497,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5">
@@ -521,7 +527,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8">
@@ -531,7 +537,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2277</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="9">
@@ -541,7 +547,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11.385</v>
+        <v>11.373</v>
       </c>
     </row>
     <row r="10">
@@ -551,7 +557,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>621.5</v>
+        <v>622</v>
       </c>
     </row>
     <row r="11">
@@ -561,7 +567,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -599,10 +605,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C15" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16">
@@ -615,7 +621,7 @@
         <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17">
@@ -625,10 +631,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" t="n">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18">
@@ -638,10 +644,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C18" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19">
@@ -654,7 +660,7 @@
         <v>8</v>
       </c>
       <c r="C19" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="20">
@@ -664,10 +670,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C20" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="21">
@@ -677,10 +683,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C21" t="n">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="22">
@@ -690,10 +696,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C22" t="n">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="23">
@@ -703,23 +709,62 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C23" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Evidence_Confidence</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Service_Conditions_Addressed</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Conceptual_Theme</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Coding_Confidence</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B27" t="n">
         <v>3</v>
       </c>
-      <c r="C24" t="n">
-        <v>200</v>
+      <c r="C27" t="n">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -733,10 +778,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -780,10 +825,10 @@
         <v>62</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>31</v>
+        <v>30.8</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -799,10 +844,10 @@
         <v>50</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -818,7 +863,7 @@
         <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
         <v>10</v>
@@ -837,7 +882,7 @@
         <v>19</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
         <v>9.5</v>
@@ -856,7 +901,7 @@
         <v>14</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
         <v>7</v>
@@ -875,7 +920,7 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
         <v>6.5</v>
@@ -894,7 +939,7 @@
         <v>8</v>
       </c>
       <c r="C8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D8" t="n">
         <v>4</v>
@@ -913,7 +958,7 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" t="n">
         <v>3.5</v>
@@ -932,7 +977,7 @@
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D10" t="n">
         <v>1.5</v>
@@ -951,7 +996,7 @@
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D11" t="n">
         <v>1.5</v>
@@ -963,14 +1008,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>pervasive_game</t>
+          <t>[tabletop_game, digital_game, escape_room_or_breakout_box, gamification]</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D12" t="n">
         <v>0.5</v>
@@ -979,8 +1024,27 @@
         <v>10</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>pervasive_game</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>201</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -991,10 +1055,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -1038,10 +1102,10 @@
         <v>99</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>49.5</v>
+        <v>49.3</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -1057,10 +1121,10 @@
         <v>77</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>38.5</v>
+        <v>38.3</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -1076,10 +1140,10 @@
         <v>56</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>28</v>
+        <v>27.9</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -1095,10 +1159,10 @@
         <v>35</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
@@ -1114,10 +1178,10 @@
         <v>29</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
@@ -1133,7 +1197,7 @@
         <v>19</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
         <v>9.5</v>
@@ -1152,7 +1216,7 @@
         <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D8" t="n">
         <v>7</v>
@@ -1171,7 +1235,7 @@
         <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" t="n">
         <v>6.5</v>
@@ -1190,7 +1254,7 @@
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D10" t="n">
         <v>2.5</v>
@@ -1209,7 +1273,7 @@
         <v>4</v>
       </c>
       <c r="C11" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D11" t="n">
         <v>2</v>
@@ -1218,8 +1282,27 @@
         <v>10</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[collections_and_access, programming_and_facilitation, learning_and_literacy, outreach_and_partnerships, professional_capacity]</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>201</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1230,7 +1313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1277,10 +1360,10 @@
         <v>123</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>61.5</v>
+        <v>61.2</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -1296,10 +1379,10 @@
         <v>51</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -1315,7 +1398,7 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
         <v>9</v>
@@ -1334,7 +1417,7 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
         <v>6.5</v>
@@ -1353,7 +1436,7 @@
         <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
         <v>4</v>
@@ -1372,7 +1455,7 @@
         <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
         <v>3.5</v>
@@ -1391,7 +1474,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D8" t="n">
         <v>3</v>
@@ -1410,7 +1493,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" t="n">
         <v>3</v>
@@ -1429,7 +1512,7 @@
         <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D10" t="n">
         <v>1.5</v>
@@ -1448,7 +1531,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D11" t="n">
         <v>0.5</v>
@@ -1460,14 +1543,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>adults</t>
+          <t>[students, educators]</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D12" t="n">
         <v>0.5</v>
@@ -1476,8 +1559,27 @@
         <v>9</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>adults</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>201</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1488,10 +1590,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -1535,10 +1637,10 @@
         <v>90</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>45</v>
+        <v>44.8</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -1554,10 +1656,10 @@
         <v>64</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>31.8</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -1573,10 +1675,10 @@
         <v>25</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>12.5</v>
+        <v>12.4</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -1592,7 +1694,7 @@
         <v>20</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
         <v>10</v>
@@ -1611,7 +1713,7 @@
         <v>17</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
         <v>8.5</v>
@@ -1630,7 +1732,7 @@
         <v>14</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
         <v>7</v>
@@ -1649,7 +1751,7 @@
         <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D8" t="n">
         <v>7</v>
@@ -1668,7 +1770,7 @@
         <v>11</v>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" t="n">
         <v>5.5</v>
@@ -1687,7 +1789,7 @@
         <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D10" t="n">
         <v>3</v>
@@ -1706,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="C11" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D11" t="n">
         <v>1.5</v>
@@ -1715,13 +1817,236 @@
         <v>9</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[equitable_access, learning_and_literacy, engagement_and_participation, institutional_capacity]</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>201</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:E12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>feature_value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>article_count</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>total_articles</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>article_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>rank_within_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>practitioner_knowledge</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>201</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>feature_value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>article_count</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>total_articles</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>article_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>rank_within_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[access_infrastructure_required, skilled_facilitation_required, inclusive_design_or_accessibility, evaluation_or_reflection]</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>201</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>feature_value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>article_count</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>total_articles</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>article_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>rank_within_group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[service_ecology, conditional_benefits]</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>201</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1771,10 +2096,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
         <v>97.5</v>
@@ -1793,7 +2118,7 @@
         <v>3</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
         <v>1.5</v>
@@ -1812,7 +2137,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -2060,10 +2385,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
@@ -2102,7 +2427,7 @@
         <v>29</v>
       </c>
       <c r="C20" t="n">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="21">
@@ -2115,7 +2440,7 @@
         <v>39</v>
       </c>
       <c r="C21" t="n">
-        <v>19.5</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="22">
@@ -2156,11 +2481,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -2214,10 +2539,10 @@
         <v>123</v>
       </c>
       <c r="D2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E2" t="n">
-        <v>61.5</v>
+        <v>61.2</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -2238,10 +2563,10 @@
         <v>51</v>
       </c>
       <c r="D3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E3" t="n">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
@@ -2262,7 +2587,7 @@
         <v>18</v>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E4" t="n">
         <v>9</v>
@@ -2286,7 +2611,7 @@
         <v>13</v>
       </c>
       <c r="D5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E5" t="n">
         <v>6.5</v>
@@ -2310,7 +2635,7 @@
         <v>8</v>
       </c>
       <c r="D6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
@@ -2334,7 +2659,7 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E7" t="n">
         <v>3.5</v>
@@ -2358,7 +2683,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
@@ -2382,7 +2707,7 @@
         <v>6</v>
       </c>
       <c r="D9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
@@ -2406,7 +2731,7 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E10" t="n">
         <v>1.5</v>
@@ -2430,7 +2755,7 @@
         <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E11" t="n">
         <v>0.5</v>
@@ -2447,14 +2772,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>adults</t>
+          <t>[students, educators]</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E12" t="n">
         <v>0.5</v>
@@ -2466,25 +2791,25 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>coding_confidence</t>
+          <t>audience</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>adults</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>195</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E13" t="n">
-        <v>97.5</v>
+        <v>0.5</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -2495,20 +2820,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>196</v>
       </c>
       <c r="D14" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E14" t="n">
-        <v>1.5</v>
+        <v>97.5</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -2519,92 +2844,92 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>201</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F15" t="n">
         <v>2</v>
-      </c>
-      <c r="D15" t="n">
-        <v>200</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>coding_confidence</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>empirical_study</t>
+          <t>low</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E16" t="n">
-        <v>39.5</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>conceptual_theme</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>practitioner_reflection</t>
+          <t>[service_ecology, conditional_benefits]</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E17" t="n">
-        <v>29</v>
+        <v>0.5</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>evidence_confidence</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>theoretical_or_conceptual</t>
+          <t>practitioner_knowledge</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>0.5</v>
       </c>
       <c r="F18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2615,20 +2940,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>implementation_case</t>
+          <t>empirical_study</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="D19" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E19" t="n">
-        <v>12</v>
+        <v>37.8</v>
       </c>
       <c r="F19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -2639,20 +2964,20 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>evidence_synthesis</t>
+          <t>practitioner_reflection</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="D20" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E20" t="n">
-        <v>6.5</v>
+        <v>18.9</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -2663,20 +2988,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>instrument_or_framework_development</t>
+          <t>theoretical_or_conceptual</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="D21" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E21" t="n">
-        <v>6.5</v>
+        <v>12.9</v>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -2687,116 +3012,116 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>content_or_artifact_analysis</t>
+          <t>implementation_case</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D22" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>11.9</v>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>digital_game</t>
+          <t>professional_practice_artifact</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="D23" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E23" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>multiple_game_formats</t>
+          <t>evidence_synthesis</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="D24" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E24" t="n">
-        <v>25</v>
+        <v>6.5</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>tabletop_game</t>
+          <t>instrument_or_framework_development</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D25" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E25" t="n">
-        <v>10</v>
+        <v>6.5</v>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>game_format</t>
+          <t>evidence_type</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>tabletop_roleplaying_game</t>
+          <t>content_or_artifact_analysis</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="D26" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E26" t="n">
-        <v>9.5</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27">
@@ -2807,20 +3132,20 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>virtual_or_augmented_reality</t>
+          <t>digital_game</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="D27" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>30.8</v>
       </c>
       <c r="F27" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -2831,20 +3156,20 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>gamification</t>
+          <t>multiple_game_formats</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="D28" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E28" t="n">
-        <v>6.5</v>
+        <v>24.9</v>
       </c>
       <c r="F28" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -2855,20 +3180,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>escape_room_or_breakout_box</t>
+          <t>tabletop_game</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D29" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
@@ -2879,20 +3204,20 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>unspecified_game_format</t>
+          <t>tabletop_roleplaying_game</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="D30" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E30" t="n">
-        <v>3.5</v>
+        <v>9.5</v>
       </c>
       <c r="F30" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -2903,20 +3228,20 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>toy_or_open_play</t>
+          <t>virtual_or_augmented_reality</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D31" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E31" t="n">
-        <v>1.5</v>
+        <v>7</v>
       </c>
       <c r="F31" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32">
@@ -2927,20 +3252,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>game_creation</t>
+          <t>gamification</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D32" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E32" t="n">
-        <v>1.5</v>
+        <v>6.5</v>
       </c>
       <c r="F32" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -2951,140 +3276,140 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>pervasive_game</t>
+          <t>escape_room_or_breakout_box</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D33" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E33" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>unspecified_game_format</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>90</v>
+        <v>7</v>
       </c>
       <c r="D34" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E34" t="n">
-        <v>45</v>
+        <v>3.5</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>learning_and_literacy</t>
+          <t>toy_or_open_play</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>64</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E35" t="n">
-        <v>32</v>
+        <v>1.5</v>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>discovery_and_advisory</t>
+          <t>game_creation</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E36" t="n">
-        <v>12.5</v>
+        <v>1.5</v>
       </c>
       <c r="F36" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>belonging_and_community</t>
+          <t>[tabletop_game, digital_game, escape_room_or_breakout_box, gamification]</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F37" t="n">
         <v>10</v>
-      </c>
-      <c r="F37" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>intended_outcome</t>
+          <t>game_format</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>creativity_and_production</t>
+          <t>pervasive_game</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E38" t="n">
-        <v>8.5</v>
+        <v>0.5</v>
       </c>
       <c r="F38" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39">
@@ -3095,20 +3420,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>institutional_capacity</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="D39" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>44.8</v>
       </c>
       <c r="F39" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -3119,20 +3444,20 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>equitable_access</t>
+          <t>learning_and_literacy</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>14</v>
+        <v>64</v>
       </c>
       <c r="D40" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>31.8</v>
       </c>
       <c r="F40" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -3143,20 +3468,20 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>engagement_and_participation</t>
+          <t>discovery_and_advisory</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="D41" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E41" t="n">
-        <v>5.5</v>
+        <v>12.4</v>
       </c>
       <c r="F41" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
@@ -3167,20 +3492,20 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>cultural_stewardship_and_preservation</t>
+          <t>belonging_and_community</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D42" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43">
@@ -3191,164 +3516,164 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>wellness_and_resilience</t>
+          <t>creativity_and_production</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D43" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E43" t="n">
-        <v>1.5</v>
+        <v>8.5</v>
       </c>
       <c r="F43" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>non_library_context</t>
+          <t>institutional_capacity</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="D44" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E44" t="n">
-        <v>23.5</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>unspecified_library_context</t>
+          <t>equitable_access</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="D45" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E45" t="n">
-        <v>23.5</v>
+        <v>7</v>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>public_library</t>
+          <t>engagement_and_participation</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D46" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E46" t="n">
-        <v>15</v>
+        <v>5.5</v>
       </c>
       <c r="F46" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>cultural_heritage_institution</t>
+          <t>cultural_stewardship_and_preservation</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="D47" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E47" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>academic_library</t>
+          <t>wellness_and_resilience</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E48" t="n">
-        <v>11</v>
+        <v>1.5</v>
       </c>
       <c r="F48" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>library_context</t>
+          <t>intended_outcome</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>multiple_library_types</t>
+          <t>[equitable_access, learning_and_literacy, engagement_and_participation, institutional_capacity]</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E49" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F49" t="n">
         <v>10</v>
-      </c>
-      <c r="F49" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="50">
@@ -3359,20 +3684,20 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>school_library</t>
+          <t>non_library_context</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="D50" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E50" t="n">
-        <v>4.5</v>
+        <v>23.4</v>
       </c>
       <c r="F50" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -3383,260 +3708,260 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>library_school</t>
+          <t>unspecified_library_context</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="D51" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E51" t="n">
-        <v>1.5</v>
+        <v>23.4</v>
       </c>
       <c r="F51" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>peer_review</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>peer_reviewed</t>
+          <t>public_library</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>116</v>
+        <v>30</v>
       </c>
       <c r="D52" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E52" t="n">
-        <v>58</v>
+        <v>14.9</v>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>peer_review</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>editorial_reviewed</t>
+          <t>academic_library</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="D53" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E53" t="n">
-        <v>19.5</v>
+        <v>11.4</v>
       </c>
       <c r="F53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>peer_review</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>cultural_heritage_institution</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D54" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E54" t="n">
-        <v>17.5</v>
+        <v>10.9</v>
       </c>
       <c r="F54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>peer_review</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>not_applicable</t>
+          <t>multiple_library_types</t>
         </is>
       </c>
       <c r="C55" t="n">
+        <v>20</v>
+      </c>
+      <c r="D55" t="n">
+        <v>201</v>
+      </c>
+      <c r="E55" t="n">
         <v>10</v>
       </c>
-      <c r="D55" t="n">
-        <v>200</v>
-      </c>
-      <c r="E55" t="n">
+      <c r="F55" t="n">
         <v>5</v>
-      </c>
-      <c r="F55" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>school_library</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="D56" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E56" t="n">
-        <v>25.5</v>
+        <v>4.5</v>
       </c>
       <c r="F56" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>library_context</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>theoretical_or_conceptual</t>
+          <t>library_school</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E57" t="n">
-        <v>14</v>
+        <v>1.5</v>
       </c>
       <c r="F57" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>peer_review</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>case_or_design_study</t>
+          <t>peer_reviewed</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="D58" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E58" t="n">
-        <v>12</v>
+        <v>57.7</v>
       </c>
       <c r="F58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>peer_review</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>mixed_methods</t>
+          <t>editorial_reviewed</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="D59" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E59" t="n">
-        <v>10.5</v>
+        <v>19.9</v>
       </c>
       <c r="F59" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>peer_review</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>qualitative_study</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D60" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E60" t="n">
-        <v>10</v>
+        <v>17.4</v>
       </c>
       <c r="F60" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>primary_methodology</t>
+          <t>peer_review</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>experimental_study</t>
+          <t>not_applicable</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D61" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="62">
@@ -3647,20 +3972,20 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>survey</t>
+          <t>none</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="D62" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E62" t="n">
-        <v>7</v>
+        <v>17.9</v>
       </c>
       <c r="F62" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -3671,20 +3996,20 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>evidence_synthesis</t>
+          <t>theoretical_or_conceptual</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D63" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E63" t="n">
-        <v>6.5</v>
+        <v>13.9</v>
       </c>
       <c r="F63" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
@@ -3695,20 +4020,20 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>content_analysis</t>
+          <t>case_or_design_study</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="D64" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>11.4</v>
       </c>
       <c r="F64" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="65">
@@ -3719,20 +4044,20 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>historical_analysis</t>
+          <t>mixed_methods</t>
         </is>
       </c>
       <c r="C65" t="n">
+        <v>21</v>
+      </c>
+      <c r="D65" t="n">
+        <v>201</v>
+      </c>
+      <c r="E65" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="F65" t="n">
         <v>4</v>
-      </c>
-      <c r="D65" t="n">
-        <v>200</v>
-      </c>
-      <c r="E65" t="n">
-        <v>2</v>
-      </c>
-      <c r="F65" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="66">
@@ -3743,20 +4068,20 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>participatory_design</t>
+          <t>community_curation</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D66" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F66" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67">
@@ -3767,188 +4092,188 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>action_research</t>
+          <t>qualitative_study</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D67" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E67" t="n">
-        <v>0.5</v>
+        <v>8.5</v>
       </c>
       <c r="F67" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>service_area</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>learning_and_literacy</t>
+          <t>experimental_study</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>99</v>
+        <v>14</v>
       </c>
       <c r="D68" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E68" t="n">
-        <v>49.5</v>
+        <v>7</v>
       </c>
       <c r="F68" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>service_area</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>collections_and_access</t>
+          <t>survey</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="D69" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E69" t="n">
-        <v>38.5</v>
+        <v>7</v>
       </c>
       <c r="F69" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>service_area</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>programming_and_facilitation</t>
+          <t>evidence_synthesis</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="D70" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E70" t="n">
-        <v>28</v>
+        <v>6.5</v>
       </c>
       <c r="F70" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>service_area</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>discovery_and_advisory</t>
+          <t>content_analysis</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="D71" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E71" t="n">
-        <v>17.5</v>
+        <v>4</v>
       </c>
       <c r="F71" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>service_area</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>community_and_inclusion</t>
+          <t>historical_analysis</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E72" t="n">
-        <v>14.5</v>
+        <v>2</v>
       </c>
       <c r="F72" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>service_area</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>professional_capacity</t>
+          <t>participatory_design</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="D73" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E73" t="n">
-        <v>9.5</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>service_area</t>
+          <t>primary_methodology</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>cultural_heritage_and_research</t>
+          <t>action_research</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D74" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E74" t="n">
-        <v>7</v>
+        <v>0.5</v>
       </c>
       <c r="F74" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="75">
@@ -3959,20 +4284,20 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>space_and_infrastructure</t>
+          <t>learning_and_literacy</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>13</v>
+        <v>99</v>
       </c>
       <c r="D75" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E75" t="n">
-        <v>6.5</v>
+        <v>49.3</v>
       </c>
       <c r="F75" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -3983,20 +4308,20 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>outreach_and_partnerships</t>
+          <t>collections_and_access</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>5</v>
+        <v>77</v>
       </c>
       <c r="D76" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E76" t="n">
-        <v>2.5</v>
+        <v>38.3</v>
       </c>
       <c r="F76" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
@@ -4007,236 +4332,236 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>creation_and_making</t>
+          <t>programming_and_facilitation</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>4</v>
+        <v>56</v>
       </c>
       <c r="D77" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E77" t="n">
-        <v>2</v>
+        <v>27.9</v>
       </c>
       <c r="F77" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>peer_reviewed_journal_article</t>
+          <t>discovery_and_advisory</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>116</v>
+        <v>35</v>
       </c>
       <c r="D78" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E78" t="n">
-        <v>58</v>
+        <v>17.4</v>
       </c>
       <c r="F78" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>toolkit_or_guidance_document</t>
+          <t>community_and_inclusion</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D79" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E79" t="n">
-        <v>15.5</v>
+        <v>14.4</v>
       </c>
       <c r="F79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>professional_publication</t>
+          <t>professional_capacity</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D80" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E80" t="n">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="F80" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>conference_paper</t>
+          <t>cultural_heritage_and_research</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D81" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E81" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="F81" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>dataset_or_archive</t>
+          <t>space_and_infrastructure</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D82" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E82" t="n">
-        <v>3</v>
+        <v>6.5</v>
       </c>
       <c r="F82" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>book_chapter</t>
+          <t>outreach_and_partnerships</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D83" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F83" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>blog_or_web_article</t>
+          <t>creation_and_making</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D84" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E84" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F84" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_area</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>dissertation_or_thesis</t>
+          <t>[collections_and_access, programming_and_facilitation, learning_and_literacy, outreach_and_partnerships, professional_capacity]</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F85" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>source_type</t>
+          <t>service_conditions_addressed</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>government_or_foundation_report</t>
+          <t>[access_infrastructure_required, skilled_facilitation_required, inclusive_design_or_accessibility, evaluation_or_reflection]</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D86" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E86" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F86" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -4247,20 +4572,20 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>peer_reviewed_journal_article</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>116</v>
       </c>
       <c r="D87" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>57.7</v>
       </c>
       <c r="F87" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -4271,24 +4596,264 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
+          <t>professional_publication</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>22</v>
+      </c>
+      <c r="D88" t="n">
+        <v>201</v>
+      </c>
+      <c r="E88" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="F88" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>professional_community_working_document</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>20</v>
+      </c>
+      <c r="D89" t="n">
+        <v>201</v>
+      </c>
+      <c r="E89" t="n">
+        <v>10</v>
+      </c>
+      <c r="F89" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>toolkit_or_guidance_document</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>11</v>
+      </c>
+      <c r="D90" t="n">
+        <v>201</v>
+      </c>
+      <c r="E90" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F90" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>conference_paper</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>9</v>
+      </c>
+      <c r="D91" t="n">
+        <v>201</v>
+      </c>
+      <c r="E91" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F91" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>dataset_or_archive</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>6</v>
+      </c>
+      <c r="D92" t="n">
+        <v>201</v>
+      </c>
+      <c r="E92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F92" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>book_chapter</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>6</v>
+      </c>
+      <c r="D93" t="n">
+        <v>201</v>
+      </c>
+      <c r="E93" t="n">
+        <v>3</v>
+      </c>
+      <c r="F93" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>blog_or_web_article</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>3</v>
+      </c>
+      <c r="D94" t="n">
+        <v>201</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F94" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>3</v>
+      </c>
+      <c r="D95" t="n">
+        <v>201</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F95" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>dissertation_or_thesis</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" t="n">
+        <v>201</v>
+      </c>
+      <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>government_or_foundation_report</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>2</v>
+      </c>
+      <c r="D97" t="n">
+        <v>201</v>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>source_type</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
           <t>unpublished_document</t>
         </is>
       </c>
-      <c r="C88" t="n">
-        <v>1</v>
-      </c>
-      <c r="D88" t="n">
-        <v>200</v>
-      </c>
-      <c r="E88" t="n">
+      <c r="C98" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" t="n">
+        <v>201</v>
+      </c>
+      <c r="E98" t="n">
         <v>0.5</v>
       </c>
-      <c r="F88" t="n">
-        <v>8</v>
+      <c r="F98" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F88"/>
+  <autoFilter ref="A1:F98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4299,10 +4864,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
   </cols>
@@ -4905,12 +5470,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>coding_confidence_matrix.csv</t>
+          <t>evidence_confidence_matrix.csv</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Binary article × Coding_Confidence matrix</t>
+          <t>Binary article × Evidence_Confidence matrix</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4922,22 +5487,124 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>evidence_confidence_counts.csv</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Aggregate counts for Evidence_Confidence</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>feature_group + feature_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>service_conditions_addressed_matrix.csv</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Binary article × Service_Conditions_Addressed matrix</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>service_conditions_addressed_counts.csv</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Aggregate counts for Service_Conditions_Addressed</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>feature_group + feature_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>conceptual_theme_matrix.csv</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Binary article × Conceptual_Theme matrix</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>conceptual_theme_counts.csv</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Aggregate counts for Conceptual_Theme</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>feature_group + feature_value</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>coding_confidence_matrix.csv</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Binary article × Coding_Confidence matrix</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>article_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>coding_confidence_counts.csv</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>Aggregate counts for Coding_Confidence</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>feature_group + feature_value</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C37"/>
+  <autoFilter ref="A1:C43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4948,10 +5615,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -4995,10 +5662,10 @@
         <v>116</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>58</v>
+        <v>57.7</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -5007,17 +5674,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>toolkit_or_guidance_document</t>
+          <t>professional_publication</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>15.5</v>
+        <v>10.9</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -5026,17 +5693,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>professional_publication</t>
+          <t>professional_community_working_document</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -5045,17 +5712,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>conference_paper</t>
+          <t>toolkit_or_guidance_document</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
@@ -5064,17 +5731,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dataset_or_archive</t>
+          <t>conference_paper</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
@@ -5083,36 +5750,36 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>book_chapter</t>
+          <t>dataset_or_archive</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>blog_or_web_article</t>
+          <t>book_chapter</t>
         </is>
       </c>
       <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>201</v>
+      </c>
+      <c r="D8" t="n">
         <v>3</v>
-      </c>
-      <c r="C8" t="n">
-        <v>200</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1.5</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
@@ -5121,17 +5788,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dissertation_or_thesis</t>
+          <t>blog_or_web_article</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -5140,17 +5807,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>government_or_foundation_report</t>
+          <t>book</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E10" t="n">
         <v>7</v>
@@ -5159,43 +5826,62 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>dissertation_or_thesis</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>unpublished_document</t>
+          <t>government_or_foundation_report</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D12" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>8</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>unpublished_document</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>201</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5253,10 +5939,10 @@
         <v>116</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>58</v>
+        <v>57.7</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -5269,13 +5955,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>19.5</v>
+        <v>19.9</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -5291,10 +5977,10 @@
         <v>35</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -5310,7 +5996,7 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
         <v>5</v>
@@ -5331,7 +6017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -5375,13 +6061,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>39.5</v>
+        <v>37.8</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -5394,13 +6080,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>29</v>
+        <v>18.9</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -5416,10 +6102,10 @@
         <v>26</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>12.9</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -5435,10 +6121,10 @@
         <v>24</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
@@ -5447,17 +6133,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>evidence_synthesis</t>
+          <t>professional_practice_artifact</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
-        <v>6.5</v>
+        <v>10</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
@@ -5466,43 +6152,62 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>instrument_or_framework_development</t>
+          <t>evidence_synthesis</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
         <v>6.5</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>content_or_artifact_analysis</t>
+          <t>instrument_or_framework_development</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="E8" t="n">
         <v>6</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>content_or_artifact_analysis</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" t="n">
+        <v>201</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:E9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5513,7 +6218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -5557,13 +6262,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>25.5</v>
+        <v>17.9</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -5579,10 +6284,10 @@
         <v>28</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>14</v>
+        <v>13.9</v>
       </c>
       <c r="E3" t="n">
         <v>2</v>
@@ -5595,13 +6300,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>11.4</v>
       </c>
       <c r="E4" t="n">
         <v>3</v>
@@ -5617,10 +6322,10 @@
         <v>21</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
@@ -5629,14 +6334,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>qualitative_study</t>
+          <t>community_curation</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
         <v>10</v>
@@ -5648,17 +6353,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>experimental_study</t>
+          <t>qualitative_study</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="E7" t="n">
         <v>6</v>
@@ -5667,36 +6372,36 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>survey</t>
+          <t>experimental_study</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>14</v>
       </c>
       <c r="C8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D8" t="n">
         <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>evidence_synthesis</t>
+          <t>survey</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="E9" t="n">
         <v>7</v>
@@ -5705,17 +6410,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>content_analysis</t>
+          <t>evidence_synthesis</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>6.5</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -5724,17 +6429,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>historical_analysis</t>
+          <t>content_analysis</t>
         </is>
       </c>
       <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>201</v>
+      </c>
+      <c r="D11" t="n">
         <v>4</v>
-      </c>
-      <c r="C11" t="n">
-        <v>200</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>9</v>
@@ -5743,17 +6448,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>participatory_design</t>
+          <t>historical_analysis</t>
         </is>
       </c>
       <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>201</v>
+      </c>
+      <c r="D12" t="n">
         <v>2</v>
-      </c>
-      <c r="C12" t="n">
-        <v>200</v>
-      </c>
-      <c r="D12" t="n">
-        <v>1</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
@@ -5762,24 +6467,43 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>action_research</t>
+          <t>participatory_design</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
         <v>11</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>action_research</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>201</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E14" t="n">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5837,10 +6561,10 @@
         <v>47</v>
       </c>
       <c r="C2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D2" t="n">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -5856,10 +6580,10 @@
         <v>47</v>
       </c>
       <c r="C3" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -5875,10 +6599,10 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>14.9</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -5887,17 +6611,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cultural_heritage_institution</t>
+          <t>academic_library</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -5906,20 +6630,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>academic_library</t>
+          <t>cultural_heritage_institution</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>22</v>
       </c>
       <c r="C6" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>10.9</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -5932,13 +6656,13 @@
         <v>20</v>
       </c>
       <c r="C7" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D7" t="n">
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -5951,13 +6675,13 @@
         <v>9</v>
       </c>
       <c r="C8" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D8" t="n">
         <v>4.5</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -5970,13 +6694,13 @@
         <v>3</v>
       </c>
       <c r="C9" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D9" t="n">
         <v>1.5</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>